<commit_message>
all excels are generated. To do: Frontend, validation, and authorization
</commit_message>
<xml_diff>
--- a/Solution1/ProjectClock.MVC/wwwroot/excel_templates/template_project.xlsx
+++ b/Solution1/ProjectClock.MVC/wwwroot/excel_templates/template_project.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Spreadsheet generated by Project clock</t>
   </si>
@@ -44,9 +44,6 @@
   </si>
   <si>
     <t>Total time</t>
-  </si>
-  <si>
-    <t>Cost per hour</t>
   </si>
   <si>
     <t>Total cost</t>
@@ -434,11 +431,9 @@
       <c r="C4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="9"/>
+      <c r="E4" s="9" t="s">
         <v>11</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5">

</xml_diff>